<commit_message>
metidos commets web profe 3a ev
</commit_message>
<xml_diff>
--- a/matematicas_1ESOA/notas/E1A_eval3.xlsx
+++ b/matematicas_1ESOA/notas/E1A_eval3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ac4744725179635e/Desktop/sapere_aude/matematicas_1ESOA/notas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="14_{58771957-A840-4041-8B91-A2D140E63AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E272A53-0A77-419D-9C24-E90131FEB078}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{B98E66C7-7952-447C-BF94-DCE475A7BE88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -703,28 +703,7 @@
     <cellStyle name="Normal 2" xfId="3" xr:uid="{9895B3A8-33B1-4097-9401-CCBAD4B00410}"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF808080"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill>
@@ -1002,6 +981,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3490,15 +3473,15 @@
     <mergeCell ref="W15:Y15"/>
   </mergeCells>
   <conditionalFormatting sqref="C2:Q26">
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="lessThan">
       <formula>5</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>LEN(TRIM(C2))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:S27">
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="5" operator="equal">
       <formula>"X"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
tabla amortizaciones hipoteca mala hecha por mi
</commit_message>
<xml_diff>
--- a/matematicas_1ESOA/notas/E1A_eval3.xlsx
+++ b/matematicas_1ESOA/notas/E1A_eval3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ac4744725179635e/Desktop/sapere_aude/matematicas_1ESOA/notas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{B98E66C7-7952-447C-BF94-DCE475A7BE88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="14_{0E956CBD-B475-4904-AA7E-6FA203F212DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4C0DC26-CD17-4B5D-8842-976D985FE556}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,8 +36,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={51B8DA1D-C762-4DCE-9FDD-3F4BEB0091B7}</author>
+  </authors>
+  <commentList>
+    <comment ref="D9" authorId="0" shapeId="0" xr:uid="{51B8DA1D-C762-4DCE-9FDD-3F4BEB0091B7}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    5 en copia jefatura</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="75">
   <si>
     <t>HOJA DE CÁLCULO PARA GENERAR UN ACTILLA DE EVALUACIÓN</t>
   </si>
@@ -433,7 +451,7 @@
       <name val="Times New Roman"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -444,6 +462,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD0CECE"/>
         <bgColor rgb="FFCCCCFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -603,7 +627,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -684,6 +708,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -984,7 +1009,9 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Eduardo Olivares López" id="{3D57B79D-55D9-4F15-A4FB-45B73F2A50C9}" userId="ac4744725179635e" providerId="Windows Live"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1282,6 +1309,14 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="D9" dT="2026-06-16T08:26:53.42" personId="{3D57B79D-55D9-4F15-A4FB-45B73F2A50C9}" id="{51B8DA1D-C762-4DCE-9FDD-3F4BEB0091B7}">
+    <text>5 en copia jefatura</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:AMK26"/>
@@ -1314,16 +1349,16 @@
       </c>
     </row>
     <row r="8" spans="2:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="35" t="s">
+      <c r="B8" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="35"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="36"/>
+      <c r="I8" s="36"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.3">
       <c r="C9" s="2" t="s">
@@ -1341,16 +1376,16 @@
       </c>
     </row>
     <row r="15" spans="2:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="35" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="35"/>
-      <c r="I15" s="35"/>
+      <c r="B15" s="36" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="36"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="36"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="36"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B17" s="2" t="s">
@@ -1373,16 +1408,16 @@
       </c>
     </row>
     <row r="22" spans="2:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="35" t="s">
+      <c r="B22" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35"/>
-      <c r="G22" s="35"/>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="36"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.3">
       <c r="N23" s="4" t="s">
@@ -1420,7 +1455,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1535,14 +1570,14 @@
       <c r="J2" s="31">
         <v>5</v>
       </c>
-      <c r="K2" s="31" t="s">
-        <v>49</v>
+      <c r="K2" s="31">
+        <v>7</v>
       </c>
       <c r="L2" s="31">
         <v>4</v>
       </c>
-      <c r="M2" s="31" t="s">
-        <v>49</v>
+      <c r="M2" s="31">
+        <v>5</v>
       </c>
       <c r="N2" s="31">
         <v>6</v>
@@ -1562,15 +1597,15 @@
       </c>
       <c r="S2" s="14" t="str">
         <f t="shared" ref="S2:S26" si="1">IF(T2&gt;$T$27,"X","")</f>
-        <v>X</v>
+        <v/>
       </c>
       <c r="T2" s="14">
         <f t="shared" ref="T2:T26" si="2">COUNTBLANK(C2:Q2)</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U2" s="15">
         <f t="shared" ref="U2:U26" si="3">(SUM(C2:Q2)+(COUNTIF(C2:Q2,"10-M")*10))/(COUNTIF(C2:Q2,"10-M")+COUNT(C2:Q2)+COUNTIF(C2:Q2,"NP")+COUNTIF(C2:Q2,"NE"))</f>
-        <v>5.375</v>
+        <v>5.5</v>
       </c>
       <c r="X2" s="16" t="s">
         <v>22</v>
@@ -1616,8 +1651,8 @@
       <c r="L3" s="31">
         <v>9</v>
       </c>
-      <c r="M3" s="31" t="s">
-        <v>49</v>
+      <c r="M3" s="31">
+        <v>9</v>
       </c>
       <c r="N3" s="31" t="s">
         <v>49</v>
@@ -1641,11 +1676,11 @@
       </c>
       <c r="T3" s="19">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U3" s="20">
         <f t="shared" si="3"/>
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="W3" s="21">
         <v>0</v>
@@ -1696,8 +1731,8 @@
       <c r="L4" s="31">
         <v>6</v>
       </c>
-      <c r="M4" s="31" t="s">
-        <v>49</v>
+      <c r="M4" s="31">
+        <v>9</v>
       </c>
       <c r="N4" s="31" t="s">
         <v>49</v>
@@ -1721,11 +1756,11 @@
       </c>
       <c r="T4" s="14">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U4" s="15">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="W4" s="24" t="s">
         <v>24</v>
@@ -1776,8 +1811,8 @@
       <c r="L5" s="31">
         <v>5</v>
       </c>
-      <c r="M5" s="31" t="s">
-        <v>49</v>
+      <c r="M5" s="31">
+        <v>4</v>
       </c>
       <c r="N5" s="31" t="s">
         <v>49</v>
@@ -1793,7 +1828,7 @@
       </c>
       <c r="R5" s="18">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S5" s="14" t="str">
         <f t="shared" si="1"/>
@@ -1801,11 +1836,11 @@
       </c>
       <c r="T5" s="19">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U5" s="20">
         <f t="shared" si="3"/>
-        <v>3.3333333333333335</v>
+        <v>3.4</v>
       </c>
       <c r="W5" s="24" t="s">
         <v>25</v>
@@ -1856,8 +1891,8 @@
       <c r="L6" s="31">
         <v>5</v>
       </c>
-      <c r="M6" s="31" t="s">
-        <v>49</v>
+      <c r="M6" s="31">
+        <v>4</v>
       </c>
       <c r="N6" s="31" t="s">
         <v>49</v>
@@ -1873,7 +1908,7 @@
       </c>
       <c r="R6" s="13">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S6" s="14" t="str">
         <f t="shared" si="1"/>
@@ -1881,11 +1916,11 @@
       </c>
       <c r="T6" s="14">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U6" s="15">
         <f t="shared" si="3"/>
-        <v>3.8888888888888888</v>
+        <v>3.9</v>
       </c>
       <c r="W6" s="24" t="s">
         <v>26</v>
@@ -1936,8 +1971,8 @@
       <c r="L7" s="31">
         <v>10</v>
       </c>
-      <c r="M7" s="31" t="s">
-        <v>49</v>
+      <c r="M7" s="31">
+        <v>9</v>
       </c>
       <c r="N7" s="31">
         <v>8</v>
@@ -1961,11 +1996,11 @@
       </c>
       <c r="T7" s="19">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U7" s="20">
         <f t="shared" si="3"/>
-        <v>8.5555555555555554</v>
+        <v>8.6</v>
       </c>
       <c r="W7" s="24" t="s">
         <v>27</v>
@@ -2059,8 +2094,8 @@
       <c r="C9" s="31">
         <v>5</v>
       </c>
-      <c r="D9" s="31">
-        <v>4</v>
+      <c r="D9" s="32">
+        <v>5</v>
       </c>
       <c r="E9" s="31">
         <v>5</v>
@@ -2103,7 +2138,7 @@
       </c>
       <c r="R9" s="18">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S9" s="14" t="str">
         <f t="shared" si="1"/>
@@ -2115,13 +2150,13 @@
       </c>
       <c r="U9" s="20">
         <f t="shared" si="3"/>
-        <v>5.3</v>
-      </c>
-      <c r="W9" s="32" t="s">
+        <v>5.4</v>
+      </c>
+      <c r="W9" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="X9" s="32"/>
-      <c r="Y9" s="32"/>
+      <c r="X9" s="33"/>
+      <c r="Y9" s="33"/>
     </row>
     <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="23">
@@ -2160,8 +2195,8 @@
       <c r="L10" s="31">
         <v>9</v>
       </c>
-      <c r="M10" s="31" t="s">
-        <v>49</v>
+      <c r="M10" s="31">
+        <v>9</v>
       </c>
       <c r="N10" s="31" t="s">
         <v>49</v>
@@ -2185,15 +2220,15 @@
       </c>
       <c r="T10" s="14">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U10" s="15">
         <f t="shared" si="3"/>
-        <v>8.3333333333333339</v>
-      </c>
-      <c r="W10" s="32"/>
-      <c r="X10" s="32"/>
-      <c r="Y10" s="32"/>
+        <v>8.4</v>
+      </c>
+      <c r="W10" s="33"/>
+      <c r="X10" s="33"/>
+      <c r="Y10" s="33"/>
     </row>
     <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="17">
@@ -2226,14 +2261,14 @@
       <c r="J11" s="31">
         <v>10</v>
       </c>
-      <c r="K11" s="31" t="s">
-        <v>49</v>
+      <c r="K11" s="31">
+        <v>9</v>
       </c>
       <c r="L11" s="31">
         <v>9</v>
       </c>
-      <c r="M11" s="31" t="s">
-        <v>49</v>
+      <c r="M11" s="31">
+        <v>10</v>
       </c>
       <c r="N11" s="31">
         <v>10</v>
@@ -2253,19 +2288,19 @@
       </c>
       <c r="S11" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>X</v>
+        <v/>
       </c>
       <c r="T11" s="19">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U11" s="20">
         <f t="shared" si="3"/>
-        <v>9</v>
-      </c>
-      <c r="W11" s="32"/>
-      <c r="X11" s="32"/>
-      <c r="Y11" s="32"/>
+        <v>9.1</v>
+      </c>
+      <c r="W11" s="33"/>
+      <c r="X11" s="33"/>
+      <c r="Y11" s="33"/>
     </row>
     <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="23">
@@ -2298,14 +2333,14 @@
       <c r="J12" s="31">
         <v>9</v>
       </c>
-      <c r="K12" s="31" t="s">
-        <v>49</v>
+      <c r="K12" s="31">
+        <v>8</v>
       </c>
       <c r="L12" s="31">
         <v>9</v>
       </c>
-      <c r="M12" s="31" t="s">
-        <v>49</v>
+      <c r="M12" s="31">
+        <v>9</v>
       </c>
       <c r="N12" s="31">
         <v>8</v>
@@ -2325,21 +2360,21 @@
       </c>
       <c r="S12" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>X</v>
+        <v/>
       </c>
       <c r="T12" s="14">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U12" s="15">
         <f t="shared" si="3"/>
-        <v>8.125</v>
-      </c>
-      <c r="W12" s="33" t="s">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="W12" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="X12" s="33"/>
-      <c r="Y12" s="33"/>
+      <c r="X12" s="34"/>
+      <c r="Y12" s="34"/>
     </row>
     <row r="13" spans="1:25" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="17">
@@ -2378,8 +2413,8 @@
       <c r="L13" s="31">
         <v>3</v>
       </c>
-      <c r="M13" s="31" t="s">
-        <v>49</v>
+      <c r="M13" s="31">
+        <v>4</v>
       </c>
       <c r="N13" s="31" t="s">
         <v>49</v>
@@ -2395,7 +2430,7 @@
       </c>
       <c r="R13" s="18">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S13" s="14" t="str">
         <f t="shared" si="1"/>
@@ -2403,15 +2438,15 @@
       </c>
       <c r="T13" s="19">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U13" s="20">
         <f t="shared" si="3"/>
-        <v>3.5555555555555554</v>
-      </c>
-      <c r="W13" s="33"/>
-      <c r="X13" s="33"/>
-      <c r="Y13" s="33"/>
+        <v>3.6</v>
+      </c>
+      <c r="W13" s="34"/>
+      <c r="X13" s="34"/>
+      <c r="Y13" s="34"/>
     </row>
     <row r="14" spans="1:25" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="23">
@@ -2450,8 +2485,8 @@
       <c r="L14" s="31">
         <v>6</v>
       </c>
-      <c r="M14" s="31" t="s">
-        <v>49</v>
+      <c r="M14" s="31">
+        <v>4</v>
       </c>
       <c r="N14" s="31" t="s">
         <v>49</v>
@@ -2467,7 +2502,7 @@
       </c>
       <c r="R14" s="13">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S14" s="14" t="str">
         <f t="shared" si="1"/>
@@ -2475,15 +2510,15 @@
       </c>
       <c r="T14" s="14">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U14" s="15">
         <f t="shared" si="3"/>
-        <v>4.8888888888888893</v>
-      </c>
-      <c r="W14" s="33"/>
-      <c r="X14" s="33"/>
-      <c r="Y14" s="33"/>
+        <v>4.8</v>
+      </c>
+      <c r="W14" s="34"/>
+      <c r="X14" s="34"/>
+      <c r="Y14" s="34"/>
     </row>
     <row r="15" spans="1:25" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="17">
@@ -2516,14 +2551,14 @@
       <c r="J15" s="31">
         <v>5</v>
       </c>
-      <c r="K15" s="31" t="s">
-        <v>49</v>
+      <c r="K15" s="31">
+        <v>6</v>
       </c>
       <c r="L15" s="31">
         <v>8</v>
       </c>
-      <c r="M15" s="31" t="s">
-        <v>49</v>
+      <c r="M15" s="31">
+        <v>7</v>
       </c>
       <c r="N15" s="31">
         <v>6</v>
@@ -2543,21 +2578,21 @@
       </c>
       <c r="S15" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>X</v>
+        <v/>
       </c>
       <c r="T15" s="19">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U15" s="20">
         <f t="shared" si="3"/>
-        <v>5.875</v>
-      </c>
-      <c r="W15" s="34" t="s">
+        <v>6</v>
+      </c>
+      <c r="W15" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="X15" s="34"/>
-      <c r="Y15" s="34"/>
+      <c r="X15" s="35"/>
+      <c r="Y15" s="35"/>
     </row>
     <row r="16" spans="1:25" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="23">
@@ -2596,8 +2631,8 @@
       <c r="L16" s="31">
         <v>7</v>
       </c>
-      <c r="M16" s="31" t="s">
-        <v>49</v>
+      <c r="M16" s="31">
+        <v>7</v>
       </c>
       <c r="N16" s="31" t="s">
         <v>49</v>
@@ -2621,11 +2656,11 @@
       </c>
       <c r="T16" s="14">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U16" s="15">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="17" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
@@ -2797,8 +2832,8 @@
       <c r="J19" s="31">
         <v>9</v>
       </c>
-      <c r="K19" s="31" t="s">
-        <v>49</v>
+      <c r="K19" s="31">
+        <v>7</v>
       </c>
       <c r="L19" s="31">
         <v>8</v>
@@ -2828,11 +2863,11 @@
       </c>
       <c r="T19" s="19">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U19" s="20">
         <f t="shared" si="3"/>
-        <v>7.7777777777777777</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="20" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
@@ -2872,8 +2907,8 @@
       <c r="L20" s="31">
         <v>5</v>
       </c>
-      <c r="M20" s="31" t="s">
-        <v>49</v>
+      <c r="M20" s="31">
+        <v>8</v>
       </c>
       <c r="N20" s="31" t="s">
         <v>49</v>
@@ -2897,11 +2932,11 @@
       </c>
       <c r="T20" s="14">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U20" s="15">
         <f t="shared" si="3"/>
-        <v>6.333333333333333</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="21" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
@@ -2935,8 +2970,8 @@
       <c r="J21" s="31">
         <v>8</v>
       </c>
-      <c r="K21" s="31" t="s">
-        <v>49</v>
+      <c r="K21" s="31">
+        <v>7</v>
       </c>
       <c r="L21" s="31">
         <v>8</v>
@@ -2966,11 +3001,11 @@
       </c>
       <c r="T21" s="19">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U21" s="20">
         <f t="shared" si="3"/>
-        <v>7.333333333333333</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="22" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
@@ -3004,14 +3039,14 @@
       <c r="J22" s="31">
         <v>9</v>
       </c>
-      <c r="K22" s="31" t="s">
-        <v>49</v>
+      <c r="K22" s="31">
+        <v>7</v>
       </c>
       <c r="L22" s="31">
         <v>9</v>
       </c>
-      <c r="M22" s="31" t="s">
-        <v>49</v>
+      <c r="M22" s="31">
+        <v>10</v>
       </c>
       <c r="N22" s="31">
         <v>10</v>
@@ -3031,15 +3066,15 @@
       </c>
       <c r="S22" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>X</v>
+        <v/>
       </c>
       <c r="T22" s="14">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U22" s="15">
         <f t="shared" si="3"/>
-        <v>8.375</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="23" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
@@ -3148,8 +3183,8 @@
       <c r="L24" s="31">
         <v>4</v>
       </c>
-      <c r="M24" s="31" t="s">
-        <v>49</v>
+      <c r="M24" s="31">
+        <v>4</v>
       </c>
       <c r="N24" s="31" t="s">
         <v>49</v>
@@ -3165,7 +3200,7 @@
       </c>
       <c r="R24" s="13">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S24" s="14" t="str">
         <f t="shared" si="1"/>
@@ -3173,11 +3208,11 @@
       </c>
       <c r="T24" s="14">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U24" s="15">
         <f t="shared" si="3"/>
-        <v>5.2222222222222223</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="25" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
@@ -3217,8 +3252,8 @@
       <c r="L25" s="31">
         <v>7</v>
       </c>
-      <c r="M25" s="31" t="s">
-        <v>49</v>
+      <c r="M25" s="31">
+        <v>8</v>
       </c>
       <c r="N25" s="31" t="s">
         <v>49</v>
@@ -3242,11 +3277,11 @@
       </c>
       <c r="T25" s="19">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U25" s="20">
         <f t="shared" si="3"/>
-        <v>6.8888888888888893</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
@@ -3280,14 +3315,14 @@
       <c r="J26" s="31">
         <v>8</v>
       </c>
-      <c r="K26" s="31" t="s">
-        <v>49</v>
+      <c r="K26" s="31">
+        <v>8</v>
       </c>
       <c r="L26" s="31">
         <v>10</v>
       </c>
-      <c r="M26" s="31" t="s">
-        <v>49</v>
+      <c r="M26" s="31">
+        <v>9</v>
       </c>
       <c r="N26" s="31">
         <v>10</v>
@@ -3307,15 +3342,15 @@
       </c>
       <c r="S26" s="14" t="str">
         <f t="shared" si="1"/>
-        <v>X</v>
+        <v/>
       </c>
       <c r="T26" s="14">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U26" s="15">
         <f t="shared" si="3"/>
-        <v>8.75</v>
+        <v>8.6999999999999993</v>
       </c>
     </row>
     <row r="27" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
@@ -3328,7 +3363,7 @@
       </c>
       <c r="D27" s="26">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E27" s="26">
         <f t="shared" si="4"/>
@@ -3364,7 +3399,7 @@
       </c>
       <c r="M27" s="26">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N27" s="26">
         <f t="shared" si="4"/>
@@ -3384,7 +3419,7 @@
       </c>
       <c r="R27" s="27">
         <f>AVERAGE(R2:R26)</f>
-        <v>1.6</v>
+        <v>1.76</v>
       </c>
       <c r="S27" s="14" t="str">
         <f>IF(T27&lt;$T$27,"X","")</f>
@@ -3392,11 +3427,11 @@
       </c>
       <c r="T27" s="28">
         <f>MODE(T2:T26)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U27" s="15">
         <f>(SUM(C2:Q26)+(COUNTIF(C2:Q26,"10-M")*10))/(COUNTIF(C2:Q26,"10-M")+COUNT(C2:Q26)+COUNTIF(C2:Q26,"NP")+COUNTIF(C2:Q26,"NE"))</f>
-        <v>6.3839285714285712</v>
+        <v>6.476</v>
       </c>
     </row>
     <row r="28" spans="1:21" ht="15.6" x14ac:dyDescent="0.3">
@@ -3409,7 +3444,7 @@
       </c>
       <c r="D28" s="29">
         <f t="shared" si="5"/>
-        <v>0.24</v>
+        <v>0.2</v>
       </c>
       <c r="E28" s="29">
         <f t="shared" si="5"/>
@@ -3435,9 +3470,9 @@
         <f t="shared" si="5"/>
         <v>0.12</v>
       </c>
-      <c r="K28" s="29" t="str">
+      <c r="K28" s="29">
         <f t="shared" si="5"/>
-        <v>--</v>
+        <v>0</v>
       </c>
       <c r="L28" s="29">
         <f t="shared" si="5"/>
@@ -3445,7 +3480,7 @@
       </c>
       <c r="M28" s="29">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="N28" s="29">
         <f t="shared" si="5"/>
@@ -3499,5 +3534,6 @@
   </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>